<commit_message>
feat(auth): implement user login, logout, and token authentication (#15)
</commit_message>
<xml_diff>
--- a/docs/requirements/07_Requirement_Traceability_Matrix.xlsx
+++ b/docs/requirements/07_Requirement_Traceability_Matrix.xlsx
@@ -531,12 +531,12 @@
       </x:c>
       <x:c r="F3" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">TBD</x:t>
+          <x:t>backend/src/routes/authRoutes.js; backend/src/controllers/authController.js; backend/src/services/authService.js; backend/src/repositories/userRepository.js; backend/src/utils/token.js; backend/src/middleware/authenticate.js</x:t>
         </x:is>
       </x:c>
       <x:c r="G3" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">UT-02; IT-02</x:t>
+          <x:t>UT-02; IT-02; TC-F03; SEC-01</x:t>
         </x:is>
       </x:c>
       <x:c r="H3" t="inlineStr">
@@ -546,7 +546,7 @@
       </x:c>
       <x:c r="I3" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Planned</x:t>
+          <x:t>Implemented - Awaiting Review</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -578,12 +578,12 @@
       </x:c>
       <x:c r="F4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">TBD</x:t>
+          <x:t>backend/src/routes/authRoutes.js; backend/src/controllers/authController.js; backend/src/services/authService.js; backend/src/services/tokenRevocationStore.js; backend/src/utils/token.js; backend/src/middleware/authenticate.js</x:t>
         </x:is>
       </x:c>
       <x:c r="G4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">UT-03; IT-03</x:t>
+          <x:t>UT-03; IT-03; TC-F04; SEC-09</x:t>
         </x:is>
       </x:c>
       <x:c r="H4" t="inlineStr">
@@ -593,7 +593,7 @@
       </x:c>
       <x:c r="I4" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Planned</x:t>
+          <x:t>Implemented - Awaiting Review</x:t>
         </x:is>
       </x:c>
     </x:row>

</xml_diff>